<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.002-04 Les fraises de Nina
Réécriture vocale example4 : éclat de fraisier, chemise qui remonte, tarte.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.002-04.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.002-04.xlsx
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nina, Victorino, papa</t>
+          <t>Nina, Victorino, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina veut assez de fraises pour une tarte. Victorino cueille avec elle. Un rire commence au robinet. Papa dit : le corps n'est pas une blague. Ils étendent la pâte, ensemble.</t>
+          <t>Une goutte tient sous une feuille. Terre noire, escargot, arrosoir vide. Sur la tige, un éclat de fraisier brille. Nina veut une tarte, maintenant. Elle saisit trop vite : les fraises tombent. Victorino arrive, chemise qui remonte. Un rire commence. Elle ferme la bouche, attend, ils cueillent. Le rouleau manque. Elle refuse de foncer. Merci vécu. La pâte colle à la chemise. Elle refuse. L'éclat de fraisier tient sur la feuille.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une fraise cache une goutte sous sa feuille. La terre est fraîche et un peu noire. Un escargot avance sur une barquette. L'arrosoir est couché, vide. Ça sent le vert et le sucre. Tu as vu la goutte, Nina ? Elle brille. Oui. Elle tient à la feuille. En ce moment, Nina soulève une feuille. La feuille est rêche et un peu poussiéreuse. Une petite bête se cache, puis part. Je veux une tarte. Avec beaucoup de fraises. On en cueille d'abord. Victorino arrive entre les rangs. Ses mains sont déjà un peu rouges. Victorino a un corps plus rond. Nina a un corps plus mince. Nina ouvre la bouche. Un petit rire commence. Le corps n'est pas une blague. On joue. On cueille. Nina ferme la bouche. On cueille. On cueille. Ils posent les fraises dans la barquette. Le bois de la barquette est rêche. Une feuille colle au poignet de Nina. Elle pique. C'est la feuille. Il en faut encore. Le plant du fond en a.</t>
+          <t>Une goutte tient sous une feuille. La terre est fraîche, un peu noire. Un escargot avance sur une barquette. L'arrosoir est couché, vide. Ça sent le vert et le sucre. Tu as vu la goutte, Nina ? Elle brille. Elle tient à la feuille ? Oui, papa. Le jardin sent le sucre, là. Oui, maman. Nina lève la feuille du fraisier. La feuille est rêche, un peu poussiéreuse. La goutte glisse dans la terre. Elle est partie. Une petite bête se cache, puis part. Sur la tige, un éclat de fraisier brille. Il brille, maman ! Tu le vois, sur la tige ? Oui, il brille. Je veux une tarte, maintenant ! Avec des fraises ? Beaucoup, papa. On en cueille d'abord ? Oui, maman. Nina saisit trop de fraises d'un coup. Les fruits glissent entre ses doigts. Ils tombent dans la terre noire. Elles sont par terre ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu, lourdes. Papa s'accroupit à la même hauteur. Tu veux la tarte avec Victorino ? Oui, papa. Tes mains sont dans les feuilles ? Oui, maman. En ce moment, Victorino arrive entre les rangs. Il a les mains un peu rouges. Tu viens ? Il se penche vers un fraisier bas. Sa chemise remonte un peu. Nina ouvre la bouche. Un petit rire commence. Oh. Nina ferme la bouche. Elle regarde la barquette. On cueille pour la tarte. Victorino ne dit rien, d'abord. Il regarde les fraisiers, puis Nina. Oui. Nina veut passer entre deux rangs. Victorino ne passe pas, trop juste. Attends. Nina reste. Elle n'avance pas. Victorino contourne le rang, sans se presser. Vous cueillez, tous les deux ? Oui, papa. Moi, le fraisier du fond. Ils posent les fraises dans la barquette. Le bois de la barquette est rêche. Une feuille colle au poignet de Nina. Elle pique. C'est la feuille ? Oui. Il en faut d'autres. Le fraisier du fond en a. L'éclat de fraisier tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une fraise cache une goutte sous sa feuille. La terre est fraîche et un peu noire. Un escargot avance sur une barquette. L'arrosoir est couché, vide. Ça sent le vert et le sucre. Tu as vu la goutte, Nina ? Elle brille. Oui. Elle tient à la feuille. En ce moment, Nina soulève une feuille. La feuille est rêche et un peu poussiéreuse. Une petite bête se cache, puis part. Je veux une tarte. Avec beaucoup de fraises. On en cueille d'abord. Victorino arrive entre les rangs. Ses mains sont déjà un peu rouges. Victorino a un corps plus rond. Nina a un corps plus mince. Nina ouvre la bouche. Un petit rire commence. Le corps n'est pas une blague. On joue. On cueille. Nina ferme la bouche. On cueille. On cueille. Ils posent les fraises dans la barquette. Le bois de la barquette est rêche. Une feuille colle au poignet de Nina. Elle pique. C'est la feuille. Il en faut encore. Le plant du fond en a.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une goutte tient sous une feuille. La terre est fraîche, un peu noire. Un escargot avance sur une barquette. L'arrosoir est couché, vide. Ça sent le vert et le sucre. Tu as vu la goutte, Nina ? Elle brille. Elle tient à la feuille ? Oui, papa. Le jardin sent le sucre, là. Oui, maman. Nina lève la feuille du fraisier. La feuille est rêche, un peu poussiéreuse. La goutte glisse dans la terre. Elle est partie. Une petite bête se cache, puis part. Sur la tige, un &lt;emphasis level="moderate"&gt;éclat de fraisier&lt;/emphasis&gt; brille. Il brille, maman ! Tu le vois, sur la tige ? Oui, il brille. Je veux une tarte, maintenant ! Avec des fraises ? Beaucoup, papa. On en cueille d'abord ? Oui, maman. Nina saisit trop de fraises d'un coup. Les fruits glissent entre ses doigts. Ils tombent dans la terre noire. Elles sont par terre ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu, lourdes. Papa s'accroupit à la même hauteur. Tu veux la tarte avec Victorino ? Oui, papa. Tes mains sont dans les feuilles ? Oui, maman. En ce moment, Victorino arrive entre les rangs. Il a les mains un peu rouges. Tu viens ? Il se penche vers un fraisier bas. Sa chemise remonte un peu. Nina ouvre la bouche. Un petit rire commence. Oh. Nina ferme la bouche. Elle regarde la barquette. On cueille pour la tarte. Victorino ne dit rien, d'abord. Il regarde les fraisiers, puis Nina. Oui. Nina veut passer entre deux rangs. Victorino ne passe pas, trop juste. Attends. Nina reste. Elle n'avance pas. Victorino contourne le rang, sans se presser. Vous cueillez, tous les deux ? Oui, papa. Moi, le fraisier du fond. Ils posent les fraises dans la barquette. Le bois de la barquette est rêche. Une feuille colle au poignet de Nina. Elle pique. C'est la feuille ? Oui. Il en faut d'autres. Le fraisier du fond en a. L'éclat de fraisier tremble, puis tient.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Ibrahim est au jardin avec papa. Nino arrive. Ils ont un ballon souple. Nino a un &lt;emphasis&gt;corps&lt;/emphasis&gt; plus rond. Ibrahim a un corps plus mince. Ibrahim ouvre la bouche. Un petit rire commence. Papa parle tout de suite. Papa dit : le corps n'est pas une blague. On joue. On reste gentils. Ibrahim ferme la bouche. Il hoche la tête. Ils se passent le ballon. L'herbe est tiède. Plus tard, ils rentrent. Dans le salon, papa sort un puzzle. Nino s'assoit. Ibrahim s'assoit. Ibrahim se souvient. Le corps n'est pas une blague. L'amitié ne dépend pas de la forme. On peut jouer. Ils cherchent les pièces du ciel. Nino trouve un nuage. Ibrahim trouve un oiseau. Ils assemblent. Papa dit encore : on joue ensemble. On ne commente pas le corps pour rabaisser. Le puzzle avance. Ibrahim offre une pièce à Nino. Nino dit merci. Ils sourient. [pause]</t>
+          <t>Une goutte tient sous une feuille. La terre est fraîche, un peu noire. Un escargot avance sur une barquette. L'arrosoir est couché, vide. Ça sent le vert et le sucre. Tu as vu la goutte, Nina ? Elle brille. Elle tient à la feuille ? Oui, papa. Le jardin sent le sucre, là. Oui, maman. Nina lève la feuille du fraisier. La feuille est rêche, un peu poussiéreuse. La goutte glisse dans la terre. Elle est partie. Une petite bête se cache, puis part. Sur la tige, un &lt;emphasis&gt;éclat de fraisier&lt;/emphasis&gt; brille. Il brille, maman ! Tu le vois, sur la tige ? Oui, il brille. Je veux une tarte, maintenant ! Avec des fraises ? Beaucoup, papa. On en cueille d'abord ? Oui, maman. Nina saisit trop de fraises d'un coup. Les fruits glissent entre ses doigts. Ils tombent dans la terre noire. Elles sont par terre ! Le sourire de Nina disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu, lourdes. Papa s'accroupit à la même hauteur. Tu veux la tarte avec Victorino ? Oui, papa. Tes mains sont dans les feuilles ? Oui, maman. En ce moment, Victorino arrive entre les rangs. Il a les mains un peu rouges. Tu viens ? Il se penche vers un fraisier bas. Sa chemise remonte un peu. Nina ouvre la bouche. Un petit rire commence. Oh. Nina ferme la bouche. Elle regarde la barquette. On cueille pour la tarte. Victorino ne dit rien, d'abord. Il regarde les fraisiers, puis Nina. Oui. Nina veut passer entre deux rangs. Victorino ne passe pas, trop juste. Attends. Nina reste. Elle n'avance pas. Victorino contourne le rang, sans se presser. Vous cueillez, tous les deux ? Oui, papa. Moi, le fraisier du fond. Ils posent les fraises dans la barquette. Le bois de la barquette est rêche. Une feuille colle au poignet de Nina. Elle pique. C'est la feuille ? Oui. Il en faut d'autres. Le fraisier du fond en a. L'éclat de fraisier tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>corps</t>
+          <t>éclat de fraisier</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,43 +1321,87 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_tarte_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une fraise cache une goutte sous sa feuille.
-narrateur|La terre est fraîche et un peu noire.
+          <t>narrateur|Une goutte tient sous une feuille.
+narrateur|La terre est fraîche, un peu noire.
 narrateur|Un escargot avance sur une barquette.
 narrateur|L'arrosoir est couché, vide.
 narrateur|Ça sent le vert et le sucre.
 papa|Tu as vu la goutte, Nina ?
 enfant-f|Elle brille.
-papa|Oui.
-papa|Elle tient à la feuille.
-narrateur|En ce moment, Nina soulève une feuille.
-narrateur|La feuille est rêche et un peu poussiéreuse.
+papa|Elle tient à la feuille ?
+enfant-f|Oui, papa.
+maman|Le jardin sent le sucre, là.
+enfant-f|Oui, maman.
+narrateur|Nina lève la feuille du fraisier.
+narrateur|La feuille est rêche, un peu poussiéreuse.
+narrateur|La goutte glisse dans la terre.
+enfant-f|Elle est partie.
 narrateur|Une petite bête se cache, puis part.
-enfant-f|Je veux une tarte.
-enfant-f|Avec beaucoup de fraises.
-papa|On en cueille d'abord.
-narrateur|Victorino arrive entre les rangs.
-narrateur|Ses mains sont déjà un peu rouges.
-narrateur|Victorino a un corps plus rond.
-narrateur|Nina a un corps plus mince.
+narrateur|Sur la tige, un éclat de fraisier brille.
+enfant-f|Il brille, maman !
+maman|Tu le vois, sur la tige ?
+enfant-f|Oui, il brille.
+enfant-f|Je veux une tarte, maintenant !
+papa|Avec des fraises ?
+enfant-f|Beaucoup, papa.
+maman|On en cueille d'abord ?
+enfant-f|Oui, maman.
+narrateur|Nina saisit trop de fraises d'un coup.
+narrateur|Les fruits glissent entre ses doigts.
+narrateur|Ils tombent dans la terre noire.
+enfant-f|Elles sont par terre !
+narrateur|Le sourire de Nina disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu, lourdes.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu veux la tarte avec Victorino ?
+enfant-f|Oui, papa.
+maman|Tes mains sont dans les feuilles ?
+enfant-f|Oui, maman.
+narrateur|En ce moment, Victorino arrive entre les rangs.
+narrateur|Il a les mains un peu rouges.
+enfant-f|Tu viens ?
+narrateur|Il se penche vers un fraisier bas.
+narrateur|Sa chemise remonte un peu.
 narrateur|Nina ouvre la bouche.
 narrateur|Un petit rire commence.
-papa|Le corps n'est pas une blague.
-papa|On joue.
-papa|On cueille.
+enfant-f|Oh.
 narrateur|Nina ferme la bouche.
-enfant-f|On cueille.
-copain|On cueille.
+narrateur|Elle regarde la barquette.
+enfant-f|On cueille pour la tarte.
+narrateur|Victorino ne dit rien, d'abord.
+narrateur|Il regarde les fraisiers, puis Nina.
+copain|Oui.
+narrateur|Nina veut passer entre deux rangs.
+narrateur|Victorino ne passe pas, trop juste.
+copain|Attends.
+narrateur|Nina reste.
+narrateur|Elle n'avance pas.
+narrateur|Victorino contourne le rang, sans se presser.
+papa|Vous cueillez, tous les deux ?
+enfant-f|Oui, papa.
+copain|Moi, le fraisier du fond.
 narrateur|Ils posent les fraises dans la barquette.
 narrateur|Le bois de la barquette est rêche.
 narrateur|Une feuille colle au poignet de Nina.
 enfant-f|Elle pique.
-papa|C'est la feuille.
-enfant-f|Il en faut encore.
-papa|Le plant du fond en a.</t>
+papa|C'est la feuille ?
+enfant-f|Oui.
+enfant-f|Il en faut d'autres.
+maman|Le fraisier du fond en a.
+narrateur|L'éclat de fraisier tremble, puis tient.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>jardin,fraisiers</t>
         </is>
       </c>
     </row>
@@ -1389,12 +1433,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Le corps n'est pas une blague. Que fait-on ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le &lt;emphasis level="moderate"&gt;corps&lt;/emphasis&gt; n'est pas une blague. Que fait-on ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Le &lt;emphasis&gt;corps&lt;/emphasis&gt; n'est pas une blague. Que fait-on ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Le &lt;emphasis&gt;corps&lt;/emphasis&gt; n'est pas une blague. Que fait-on ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1457,18 +1501,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1483,11 +1527,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1498,23 +1542,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1523,23 +1567,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_ferme_la_bouche_ils_cueillent; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1572,17 +1616,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Au robinet, l'eau est froide. Les fraises deviennent plus brillantes. Une goutte mouille la chemise de Victorino. Elle est froide. On rit de l'eau. On joue. Dans la cuisine, la pâte attend. Elle est molle et un peu collante. On l'étale. Moi le rouleau. Victorino tient un bout. Nina tient l'autre bout. La pâte devient un tapis. Nina pose les fraises. Elles font un petit cercle rouge. Victorino en pose aussi. Bravo, Nina. Tu as rempli la tarte. Vous jouez. L'amitié ne dépend pas de la forme. Papa met la tarte au chaud. La porte du four fait un petit clac. Elle va sentir bon. Très bon.</t>
+          <t>Au robinet, l'eau est froide. Les fraises deviennent plus brillantes. Une goutte mouille la chemise de Victorino. Elle est froide. L'eau pique les mains. Ils rient de l'eau. Elle est froide, cette goutte ? Oui, papa. On rentre pour la pâte ? Oui, maman. Dans la cuisine, la pâte attend. Elle est molle et un peu collante. On l'étale, maintenant ! Moi le rouleau. Le rouleau n'est pas sur la table. Il manque ! Nina étale avec les mains, trop vite. La pâte se déchire d'un côté. Elle est trouée. Le sourire de Nina ne revient pas. Nina refuse de foncer, cette fois. Personne ne dit la suite à voix haute. Elle regarde la barquette. Une feuille de fraisier est restée dessus. Sur la tige, l'éclat de fraisier brille. Le rouleau, papa ? Tu le cherches où ? Près de l'eau. Le rouleau attend près de l'évier. Nina l'apporte, sans se presser. Victorino tient un bout de pâte. Nina tient l'autre bout. La pâte devient un tapis. Tu tiens ce bord ? Victorino ne dit rien. Il pose une main sur la pâte, sans parler. Oui. Nina pose les fraises, une par une. Elles font un petit cercle rouge. Le milieu reste vide. Il manque le centre. J'en ai une. Victorino pose la dernière fraise au milieu. Merci, Nina. Papa a vu les deux mains sur la pâte. Victorino, tu as vu le cercle ? Oui. Un autre tour de rouleau ? Oui, papa. Le ventre de Nina se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Au robinet, l'eau est froide. Les fraises deviennent plus brillantes. Une goutte mouille la chemise de Victorino. Elle est froide. On rit de l'eau. On joue. Dans la cuisine, la pâte attend. Elle est molle et un peu collante. On l'étale. Moi le rouleau. Victorino tient un bout. Nina tient l'autre bout. La pâte devient un tapis. Nina pose les fraises. Elles font un petit cercle rouge. Victorino en pose aussi. Bravo, Nina. Tu as rempli la tarte. Vous jouez. L'amitié ne dépend pas de la forme. Papa met la tarte au chaud. La porte du four fait un petit clac. Elle va sentir bon. Très bon.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Au robinet, l'eau est froide. Les fraises deviennent plus brillantes. Une goutte mouille la chemise de Victorino. Elle est froide. L'eau pique les mains. Ils rient de l'eau. Elle est froide, cette goutte ? Oui, papa. On rentre pour la pâte ? Oui, maman. Dans la cuisine, la pâte attend. Elle est molle et un peu collante. On l'étale, maintenant ! Moi le &lt;emphasis level="moderate"&gt;rouleau&lt;/emphasis&gt;. Le rouleau n'est pas sur la table. Il manque ! Nina étale avec les mains, trop vite. La pâte se déchire d'un côté. Elle est trouée. Le sourire de Nina ne revient pas. Nina refuse de foncer, cette fois. Personne ne dit la suite à voix haute. Elle regarde la barquette. Une feuille de fraisier est restée dessus. Sur la tige, l'éclat de fraisier brille. Le rouleau, papa ? Tu le cherches où ? Près de l'eau. Le rouleau attend près de l'évier. Nina l'apporte, sans se presser. Victorino tient un bout de pâte. Nina tient l'autre bout. La pâte devient un tapis. Tu tiens ce bord ? Victorino ne dit rien. Il pose une main sur la pâte, sans parler. Oui. Nina pose les fraises, une par une. Elles font un petit cercle rouge. Le milieu reste vide. Il manque le centre. J'en ai une. Victorino pose la dernière fraise au milieu. Merci, Nina. Papa a vu les deux mains sur la pâte. Victorino, tu as vu le cercle ? Oui. Un autre tour de rouleau ? Oui, papa. Le ventre de Nina se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Ibrahim a entendu papa. Le &lt;emphasis&gt;corps&lt;/emphasis&gt; n'est pas une blague. Ibrahim et Nino ont joué. Au jardin, puis au salon. [pause]</t>
+          <t>Au robinet, l'eau est froide. Les fraises deviennent plus brillantes. Une goutte mouille la chemise de Victorino. Elle est froide. L'eau pique les mains. Ils rient de l'eau. Elle est froide, cette goutte ? Oui, papa. On rentre pour la pâte ? Oui, maman. Dans la cuisine, la pâte attend. Elle est molle et un peu collante. On l'étale, maintenant ! Moi le &lt;emphasis&gt;rouleau&lt;/emphasis&gt;. Le rouleau n'est pas sur la table. Il manque ! Nina étale avec les mains, trop vite. La pâte se déchire d'un côté. Elle est trouée. Le sourire de Nina ne revient pas. Nina refuse de foncer, cette fois. Personne ne dit la suite à voix haute. Elle regarde la barquette. Une feuille de fraisier est restée dessus. Sur la tige, l'éclat de fraisier brille. Le rouleau, papa ? Tu le cherches où ? Près de l'eau. Le rouleau attend près de l'évier. Nina l'apporte, sans se presser. Victorino tient un bout de pâte. Nina tient l'autre bout. La pâte devient un tapis. Tu tiens ce bord ? Victorino ne dit rien. Il pose une main sur la pâte, sans parler. Oui. Nina pose les fraises, une par une. Elles font un petit cercle rouge. Le milieu reste vide. Il manque le centre. J'en ai une. Victorino pose la dernière fraise au milieu. Merci, Nina. Papa a vu les deux mains sur la pâte. Victorino, tu as vu le cercle ? Oui. Un autre tour de rouleau ? Oui, papa. Le ventre de Nina se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1629,7 +1673,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1637,10 +1681,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1663,30 +1707,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>corps</t>
+          <t>rouleau</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1695,10 +1739,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1711,7 +1755,7 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_attend_trouve_le_rouleau; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
@@ -1720,26 +1764,57 @@
 narrateur|Les fraises deviennent plus brillantes.
 narrateur|Une goutte mouille la chemise de Victorino.
 copain|Elle est froide.
-papa|On rit de l'eau.
-papa|On joue.
+enfant-f|L'eau pique les mains.
+narrateur|Ils rient de l'eau.
+papa|Elle est froide, cette goutte ?
+enfant-f|Oui, papa.
+maman|On rentre pour la pâte ?
+enfant-f|Oui, maman.
 narrateur|Dans la cuisine, la pâte attend.
 narrateur|Elle est molle et un peu collante.
-enfant-f|On l'étale.
+enfant-f|On l'étale, maintenant !
 copain|Moi le rouleau.
-narrateur|Victorino tient un bout.
+narrateur|Le rouleau n'est pas sur la table.
+enfant-f|Il manque !
+narrateur|Nina étale avec les mains, trop vite.
+narrateur|La pâte se déchire d'un côté.
+enfant-f|Elle est trouée.
+narrateur|Le sourire de Nina ne revient pas.
+narrateur|Nina refuse de foncer, cette fois.
+narrateur|Personne ne dit la suite à voix haute.
+narrateur|Elle regarde la barquette.
+narrateur|Une feuille de fraisier est restée dessus.
+narrateur|Sur la tige, l'éclat de fraisier brille.
+enfant-f|Le rouleau, papa ?
+papa|Tu le cherches où ?
+enfant-f|Près de l'eau.
+narrateur|Le rouleau attend près de l'évier.
+narrateur|Nina l'apporte, sans se presser.
+narrateur|Victorino tient un bout de pâte.
 narrateur|Nina tient l'autre bout.
 narrateur|La pâte devient un tapis.
-narrateur|Nina pose les fraises.
+enfant-f|Tu tiens ce bord ?
+narrateur|Victorino ne dit rien.
+narrateur|Il pose une main sur la pâte, sans parler.
+copain|Oui.
+narrateur|Nina pose les fraises, une par une.
 narrateur|Elles font un petit cercle rouge.
-narrateur|Victorino en pose aussi.
-papa|Bravo, Nina.
-papa|Tu as rempli la tarte.
-papa|Vous jouez.
-papa|L'amitié ne dépend pas de la forme.
-narrateur|Papa met la tarte au chaud.
-narrateur|La porte du four fait un petit clac.
-enfant-f|Elle va sentir bon.
-copain|Très bon.</t>
+narrateur|Le milieu reste vide.
+enfant-f|Il manque le centre.
+copain|J'en ai une.
+narrateur|Victorino pose la dernière fraise au milieu.
+papa|Merci, Nina.
+narrateur|Papa a vu les deux mains sur la pâte.
+maman|Victorino, tu as vu le cercle ?
+copain|Oui.
+papa|Un autre tour de rouleau ?
+enfant-f|Oui, papa.
+narrateur|Le ventre de Nina se desserre.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>robinet,pate</t>
         </is>
       </c>
     </row>
@@ -1766,17 +1841,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ils attendent près de la fenêtre. Dehors, l'escargot a avancé. Il va loin. Tout doux, comme nous. Tu as fini d'attendre un moment ? Oui, papa. La tarte sort. Ça sent le sucre chaud. Le bord est un peu doré. Nina souffle un peu. Victorino souffle aussi. On goûte le bord ? Oui. C'est doux. Encore un peu. Merci d'avoir cueilli.</t>
+          <t>Nina veut la tarte au chaud, d'un coup. Elle pousse le moule trop vite. La pâte glisse d'un bord. Ça tombe ! Attends. De la pâte colle à la chemise de Victorino. Nina ouvre la bouche. Un petit rire revient, presque. Nina refuse de foncer, cette fois. Ses épaules se serrent un peu. Ça tape fort, dans sa poitrine. Personne ne dit la suite à voix haute. Elle regarde la feuille, sur la table. L'éclat de fraisier revient, sur la feuille. L'éclat, papa ? Tu le vois, toi ? Oui, sur la feuille. La tarte, Nina ? Oui. Nina attend que la pâte tienne. Victorino tient le bord, sans parler. Ils poussent le moule, sans se presser. La porte du four fait un petit clac. C'est passé. Oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Ils attendent près de la fenêtre. Dehors, l'escargot a avancé. Il va loin. Tout doux, comme nous. Tu as fini d'attendre un moment ? Oui, papa. La tarte sort. Ça sent le sucre chaud. Le bord est un peu doré. Nina souffle un peu. Victorino souffle aussi. On goûte le bord ? Oui. C'est doux. Encore un peu. Merci d'avoir cueilli.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nina veut la tarte au chaud, d'un coup. Elle pousse le moule trop vite. La pâte glisse d'un bord. Ça tombe ! Attends. De la pâte colle à la chemise de Victorino. Nina ouvre la bouche. Un petit rire revient, presque. Nina refuse de foncer, cette fois. Ses épaules se serrent un peu. Ça tape fort, dans sa poitrine. Personne ne dit la suite à voix haute. Elle regarde la feuille, sur la table. L'&lt;emphasis level="moderate"&gt;éclat de fraisier&lt;/emphasis&gt; revient, sur la feuille. L'éclat, papa ? Tu le vois, toi ? Oui, sur la feuille. La tarte, Nina ? Oui. Nina attend que la pâte tienne. Victorino tient le bord, sans parler. Ils poussent le moule, sans se presser. La porte du four fait un petit clac. C'est passé. Oui.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Papa range la boîte. Ibrahim et Nino se disent merci. [pause]</t>
+          <t>&lt;low-pitch&gt;Nina veut la tarte au chaud, d'un coup. Elle pousse le moule trop vite. La pâte glisse d'un bord. Ça tombe ! Attends. De la pâte colle à la chemise de Victorino. Nina ouvre la bouche. Un petit rire revient, presque. Nina refuse de foncer, cette fois. Ses épaules se serrent un peu. Ça tape fort, dans sa poitrine. Personne ne dit la suite à voix haute. Elle regarde la feuille, sur la table. L'&lt;emphasis&gt;éclat de fraisier&lt;/emphasis&gt; revient, sur la feuille. L'éclat, papa ? Tu le vois, toi ? Oui, sur la feuille. La tarte, Nina ? Oui. Nina attend que la pâte tienne. Victorino tient le bord, sans parler. Ils poussent le moule, sans se presser. La porte du four fait un petit clac. C'est passé. Oui.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1823,7 +1898,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1831,22 +1906,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1855,28 +1934,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de fraisier</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1885,39 +1968,57 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Ils attendent près de la fenêtre.
-narrateur|Dehors, l'escargot a avancé.
-enfant-f|Il va loin.
-papa|Tout doux, comme nous.
-papa|Tu as fini d'attendre un moment ?
-enfant-f|Oui, papa.
-narrateur|La tarte sort.
-narrateur|Ça sent le sucre chaud.
-narrateur|Le bord est un peu doré.
-narrateur|Nina souffle un peu.
-narrateur|Victorino souffle aussi.
-papa|On goûte le bord ?
-copain|Oui.
-enfant-f|C'est doux.
-copain|Encore un peu.
-papa|Merci d'avoir cueilli.</t>
+          <t>narrateur|Nina veut la tarte au chaud, d'un coup.
+narrateur|Elle pousse le moule trop vite.
+narrateur|La pâte glisse d'un bord.
+enfant-f|Ça tombe !
+copain|Attends.
+narrateur|De la pâte colle à la chemise de Victorino.
+narrateur|Nina ouvre la bouche.
+narrateur|Un petit rire revient, presque.
+narrateur|Nina refuse de foncer, cette fois.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Ça tape fort, dans sa poitrine.
+narrateur|Personne ne dit la suite à voix haute.
+narrateur|Elle regarde la feuille, sur la table.
+narrateur|L'éclat de fraisier revient, sur la feuille.
+enfant-f|L'éclat, papa ?
+papa|Tu le vois, toi ?
+enfant-f|Oui, sur la feuille.
+maman|La tarte, Nina ?
+enfant-f|Oui.
+narrateur|Nina attend que la pâte tienne.
+narrateur|Victorino tient le bord, sans parler.
+narrateur|Ils poussent le moule, sans se presser.
+narrateur|La porte du four fait un petit clac.
+enfant-f|C'est passé.
+copain|Oui.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>four,tarte</t>
         </is>
       </c>
     </row>
@@ -1944,17 +2045,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>On a fait la tarte. Avec les fraises. Vous avez joué. Une feuille de fraisier tremble encore.</t>
+          <t>Ils attendent près de la fenêtre. Dehors, l'escargot a avancé. Il va loin, papa. Tu le vois sur le bois ? Oui, papa. On est bien, ici. La tarte sort. Ça sent le sucre chaud. Le bord est un peu doré. On goûte le bord ? Vous soufflez un peu ? Oui, maman. Nina souffle. Victorino souffle aussi. C'est doux. La tarte est là. Elle est là, Nina. Oui, maman. Nina pose la joue près de la feuille. La feuille est tiède, un peu. L'éclat est là, papa. Tu le vois sur la feuille ? Oui, papa. L'éclat de fraisier tient sur la feuille.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>On a fait la tarte. Avec les fraises. Vous avez joué. Une feuille de fraisier tremble encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils attendent près de la fenêtre. Dehors, l'escargot a avancé. Il va loin, papa. Tu le vois sur le bois ? Oui, papa. On est bien, ici. La tarte sort. Ça sent le sucre chaud. Le bord est un peu doré. On goûte le bord ? Vous soufflez un peu ? Oui, maman. Nina souffle. Victorino souffle aussi. C'est doux. La tarte est là. Elle est là, Nina. Oui, maman. Nina pose la joue près de la feuille. La feuille est tiède, un peu. L'éclat est là, papa. Tu le vois sur la feuille ? Oui, papa. L'&lt;emphasis level="moderate"&gt;éclat de fraisier&lt;/emphasis&gt; tient sur la feuille.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils attendent près de la fenêtre. Dehors, l'escargot a avancé. Il va loin, papa. Tu le vois sur le bois ? Oui, papa. On est bien, ici. La tarte sort. Ça sent le sucre chaud. Le bord est un peu doré. On goûte le bord ? Vous soufflez un peu ? Oui, maman. Nina souffle. Victorino souffle aussi. C'est doux. La tarte est là. Elle est là, Nina. Oui, maman. Nina pose la joue près de la feuille. La feuille est tiède, un peu. L'éclat est là, papa. Tu le vois sur la feuille ? Oui, papa. L'&lt;emphasis&gt;éclat de fraisier&lt;/emphasis&gt; tient sur la feuille.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2001,7 +2102,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2009,10 +2110,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.12</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2021,12 +2122,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2035,17 +2136,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de fraisier</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2054,11 +2159,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2067,27 +2172,56 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_la_feuille; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|On a fait la tarte.
-copain|Avec les fraises.
-papa|Vous avez joué.
-narrateur|Une feuille de fraisier tremble encore.</t>
+          <t>narrateur|Ils attendent près de la fenêtre.
+narrateur|Dehors, l'escargot a avancé.
+enfant-f|Il va loin, papa.
+papa|Tu le vois sur le bois ?
+enfant-f|Oui, papa.
+maman|On est bien, ici.
+narrateur|La tarte sort.
+narrateur|Ça sent le sucre chaud.
+narrateur|Le bord est un peu doré.
+enfant-f|On goûte le bord ?
+maman|Vous soufflez un peu ?
+enfant-f|Oui, maman.
+narrateur|Nina souffle.
+narrateur|Victorino souffle aussi.
+copain|C'est doux.
+enfant-f|La tarte est là.
+maman|Elle est là, Nina.
+enfant-f|Oui, maman.
+narrateur|Nina pose la joue près de la feuille.
+narrateur|La feuille est tiède, un peu.
+enfant-f|L'éclat est là, papa.
+papa|Tu le vois sur la feuille ?
+enfant-f|Oui, papa.
+narrateur|L'éclat de fraisier tient sur la feuille.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>tarte</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2193,6 +2327,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>